<commit_message>
merge data with results and ground truth for evalution
</commit_message>
<xml_diff>
--- a/Invoice_100_Test/Ground_Truth/ground_truth.xlsx
+++ b/Invoice_100_Test/Ground_Truth/ground_truth.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\Invoice_100_Test\PDFs\Ground_Truth\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\AI_Invoice_Processing_Automation\Invoice_100_Test\Ground_Truth\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D27693CA-8387-40A3-840C-2E752063245E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA8C4F89-CB48-4FB6-BED4-B6C5632B791D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -525,7 +525,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J66"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="9.54296875" bestFit="1" customWidth="1"/>
@@ -731,163 +731,163 @@
         <v>16</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A62" t="s">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>37</v>
       </c>
-      <c r="B62" t="s">
+      <c r="B7" t="s">
         <v>38</v>
       </c>
-      <c r="C62" t="s">
-        <v>42</v>
-      </c>
-      <c r="D62" t="s">
+      <c r="C7" t="s">
+        <v>42</v>
+      </c>
+      <c r="D7" t="s">
         <v>39</v>
       </c>
-      <c r="E62">
+      <c r="E7">
         <v>83876203</v>
       </c>
-      <c r="F62" t="s">
+      <c r="F7" t="s">
         <v>40</v>
       </c>
-      <c r="G62">
+      <c r="G7">
         <v>280.32</v>
       </c>
-      <c r="H62" t="s">
+      <c r="H7" t="s">
         <v>41</v>
       </c>
-      <c r="I62" t="s">
-        <v>15</v>
-      </c>
-      <c r="J62" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A63" t="s">
+      <c r="I7" t="s">
+        <v>15</v>
+      </c>
+      <c r="J7" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>43</v>
       </c>
-      <c r="B63" t="s">
+      <c r="B8" t="s">
         <v>44</v>
       </c>
-      <c r="C63" t="s">
-        <v>42</v>
-      </c>
-      <c r="D63" t="s">
+      <c r="C8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D8" t="s">
         <v>45</v>
       </c>
-      <c r="E63">
+      <c r="E8">
         <v>87655538</v>
       </c>
-      <c r="F63" t="s">
+      <c r="F8" t="s">
         <v>46</v>
       </c>
-      <c r="G63">
+      <c r="G8">
         <v>853.56</v>
       </c>
-      <c r="H63" t="s">
+      <c r="H8" t="s">
         <v>41</v>
       </c>
-      <c r="I63" t="s">
-        <v>15</v>
-      </c>
-      <c r="J63" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A64" t="s">
+      <c r="I8" t="s">
+        <v>15</v>
+      </c>
+      <c r="J8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>47</v>
       </c>
-      <c r="B64" t="s">
+      <c r="B9" t="s">
         <v>48</v>
       </c>
-      <c r="C64" t="s">
-        <v>42</v>
-      </c>
-      <c r="D64" t="s">
+      <c r="C9" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" t="s">
         <v>49</v>
       </c>
-      <c r="E64">
+      <c r="E9">
         <v>37959814</v>
       </c>
-      <c r="F64" s="2">
+      <c r="F9" s="2">
         <v>41615</v>
       </c>
-      <c r="G64">
+      <c r="G9">
         <v>7285.98</v>
       </c>
-      <c r="H64" t="s">
+      <c r="H9" t="s">
         <v>41</v>
       </c>
-      <c r="I64" t="s">
-        <v>15</v>
-      </c>
-      <c r="J64" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A65" t="s">
+      <c r="I9" t="s">
+        <v>15</v>
+      </c>
+      <c r="J9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>50</v>
       </c>
-      <c r="B65" t="s">
+      <c r="B10" t="s">
         <v>51</v>
       </c>
-      <c r="C65" t="s">
-        <v>42</v>
-      </c>
-      <c r="D65" t="s">
+      <c r="C10" t="s">
+        <v>42</v>
+      </c>
+      <c r="D10" t="s">
         <v>52</v>
       </c>
-      <c r="E65">
+      <c r="E10">
         <v>37995856</v>
       </c>
-      <c r="F65" s="2">
+      <c r="F10" s="2">
         <v>42861</v>
       </c>
-      <c r="G65">
+      <c r="G10">
         <v>87.98</v>
       </c>
-      <c r="H65" t="s">
+      <c r="H10" t="s">
         <v>41</v>
       </c>
-      <c r="I65" t="s">
-        <v>15</v>
-      </c>
-      <c r="J65" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A66" t="s">
+      <c r="I10" t="s">
+        <v>15</v>
+      </c>
+      <c r="J10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
         <v>53</v>
       </c>
-      <c r="B66" t="s">
+      <c r="B11" t="s">
         <v>54</v>
       </c>
-      <c r="C66" t="s">
-        <v>42</v>
-      </c>
-      <c r="D66" t="s">
+      <c r="C11" t="s">
+        <v>42</v>
+      </c>
+      <c r="D11" t="s">
         <v>55</v>
       </c>
-      <c r="E66">
+      <c r="E11">
         <v>93128666</v>
       </c>
-      <c r="F66" t="s">
+      <c r="F11" t="s">
         <v>56</v>
       </c>
-      <c r="G66">
+      <c r="G11">
         <v>64.319999999999993</v>
       </c>
-      <c r="H66" t="s">
+      <c r="H11" t="s">
         <v>41</v>
       </c>
-      <c r="I66" t="s">
-        <v>15</v>
-      </c>
-      <c r="J66" t="s">
+      <c r="I11" t="s">
+        <v>15</v>
+      </c>
+      <c r="J11" t="s">
         <v>42</v>
       </c>
     </row>

</xml_diff>